<commit_message>
New south korea data from partners + csv export
</commit_message>
<xml_diff>
--- a/InputData/bldgs/EoDSDwSP/Elasticity of Dist Solar Deployment wrt Subsidy Perc.xlsx
+++ b/InputData/bldgs/EoDSDwSP/Elasticity of Dist Solar Deployment wrt Subsidy Perc.xlsx
@@ -1,27 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipI\InputData\bldgs\EoDSDwSP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\administer\Dropbox\kjh\2025\02. EPS\EI\251020_메일회신\회신용 파일\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDDE2B77-9DC7-43D0-B0C7-D331A5FB5BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="75" windowWidth="24915" windowHeight="12090"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Calculations" sheetId="3" r:id="rId2"/>
     <sheet name="EoDSDwSP" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Source:</t>
   </si>
@@ -85,19 +99,29 @@
   <si>
     <t>Elasticity (dimensionless)</t>
   </si>
+  <si>
+    <t>Since precise statistics are unavailable, adopt the U.S. data by referencing past cases where aggressive support policies significantly expanded domestic PV penetration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note of Korea Data: </t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://test.hri.co.kr/kor/report/report-view.html?mode=4&amp;uid=15265&amp;search=&amp;page=397</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="176" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -105,15 +129,31 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -138,7 +178,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -149,11 +189,12 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="백분율" xfId="1" builtinId="5"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -169,9 +210,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -209,9 +250,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -246,7 +287,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -281,7 +322,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -454,16 +495,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -471,59 +512,75 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" s="2">
         <v>2015</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
     </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="35.140625" customWidth="1"/>
-    <col min="3" max="3" width="45.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="35.125" customWidth="1"/>
+    <col min="3" max="3" width="45.375" customWidth="1"/>
+    <col min="4" max="4" width="22.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -537,7 +594,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -552,7 +609,7 @@
         <v>0.43949044585987279</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -567,12 +624,12 @@
         <v>0.37984496124031009</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>0.3</v>
       </c>
@@ -580,12 +637,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -594,7 +651,7 @@
         <v>1.4649681528662426</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -604,28 +661,29 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="22.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -634,7 +692,7 @@
         <v>1.4649681528662426</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -643,7 +701,7 @@
         <v>1.4649681528662426</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -653,11 +711,21 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -801,15 +869,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -817,13 +876,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33ABAF6F-4A7A-4EA0-8105-5D600EC18519}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A8269B0-4DEE-42CF-A1D2-76C3BE659685}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A8269B0-4DEE-42CF-A1D2-76C3BE659685}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33ABAF6F-4A7A-4EA0-8105-5D600EC18519}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39DCB46C-0742-4603-A7BF-23FDE354CD77}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39DCB46C-0742-4603-A7BF-23FDE354CD77}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>